<commit_message>
feat(importer): Ensure 100% consistency between green Download Sale File button output, importer parser, and Publish/260829/importfiles/ templates
</commit_message>
<xml_diff>
--- a/Publish/260829/importfiles/ExcelSample1_ExcursionSales_Import.xlsx
+++ b/Publish/260829/importfiles/ExcelSample1_ExcursionSales_Import.xlsx
@@ -398,169 +398,286 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:D12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Tour Code</v>
+        <v>Dates</v>
       </c>
       <c r="B1" t="str">
-        <v>Excursion Name</v>
+        <v>06.07.2026</v>
       </c>
       <c r="C1" t="str">
-        <v>Passenger Name</v>
+        <v>08.07.2026</v>
       </c>
       <c r="D1" t="str">
-        <v>Adult Count</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Child Count</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Sale Price (€)</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Total Amount (€)</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Payment Method</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Notes</v>
+        <v>10.07.2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BVP05072026</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Prague Castle Guided Tour</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Ahmet Yılmaz</v>
+        <v>Prices</v>
+      </c>
+      <c r="B2">
+        <v>25</v>
+      </c>
+      <c r="C2">
+        <v>45</v>
       </c>
       <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>25</v>
-      </c>
-      <c r="G2">
-        <v>50</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Cash (EUR)</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Paid to guide</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BVP05072026</v>
+        <v>Code</v>
       </c>
       <c r="B3" t="str">
+        <v>PRG-CASTLE</v>
+      </c>
+      <c r="C3" t="str">
+        <v>BUD-CRUISE</v>
+      </c>
+      <c r="D3" t="str">
+        <v>VIE-SCHONBRUNN</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Passenger Name</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Prague Castle Guided Tour</v>
+      </c>
+      <c r="C4" t="str">
         <v>Budapest Danube Dinner Cruise</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D4" t="str">
+        <v>Schönbrunn Palace Tour</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Ahmet Yılmaz</v>
+      </c>
+      <c r="B5" t="str">
+        <v>☑</v>
+      </c>
+      <c r="C5" t="str">
+        <v>☑</v>
+      </c>
+      <c r="D5" t="str">
+        <v>☐</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Ayşe Yılmaz</v>
+      </c>
+      <c r="B6" t="str">
+        <v>☑</v>
+      </c>
+      <c r="C6" t="str">
+        <v>☑</v>
+      </c>
+      <c r="D6" t="str">
+        <v>☐</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Mehmet Kaya</v>
       </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>45</v>
-      </c>
-      <c r="G3">
-        <v>115</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Credit Card</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Family ticket with 1 child</v>
+      <c r="B7" t="str">
+        <v>☐</v>
+      </c>
+      <c r="C7" t="str">
+        <v>☑</v>
+      </c>
+      <c r="D7" t="str">
+        <v>☑</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Fatma Kaya</v>
+      </c>
+      <c r="B8" t="str">
+        <v>☐</v>
+      </c>
+      <c r="C8" t="str">
+        <v>☑</v>
+      </c>
+      <c r="D8" t="str">
+        <v>☑</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Can Kaya (CHD)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>☐</v>
+      </c>
+      <c r="C9" t="str">
+        <v>☑</v>
+      </c>
+      <c r="D9" t="str">
+        <v>☑</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Count</v>
+      </c>
+      <c r="B11" t="str">
+        <v>=COUNTIF(B5:B9, "☑") + COUNTIF(B5:B9, TRUE)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>=COUNTIF(C5:C9, "☑") + COUNTIF(C5:C9, TRUE)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>=COUNTIF(D5:D9, "☑") + COUNTIF(D5:D9, TRUE)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Total Amount</v>
+      </c>
+      <c r="B12" t="str">
+        <v>=B11*B2</v>
+      </c>
+      <c r="C12" t="str">
+        <v>=C11*C2</v>
+      </c>
+      <c r="D12" t="str">
+        <v>=D11*D2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:J3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Tour Code</v>
+        <v>Base Service</v>
       </c>
       <c r="B1" t="str">
-        <v>Service Category</v>
+        <v>Revenue</v>
       </c>
       <c r="C1" t="str">
-        <v>Description</v>
+        <v>Expense</v>
       </c>
       <c r="D1" t="str">
-        <v>Quantity</v>
+        <v>Other</v>
       </c>
       <c r="E1" t="str">
-        <v>Unit Price (€)</v>
+        <v>per/Pax</v>
       </c>
       <c r="F1" t="str">
-        <v>Total Amount (€)</v>
+        <v>UnitPrice</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Adult</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Children</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Infant</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Total</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BVP05072026</v>
+        <v>Agency Fee</v>
       </c>
       <c r="B2" t="str">
-        <v>Guide</v>
+        <v>☑</v>
       </c>
       <c r="C2" t="str">
-        <v>Professional Licensed Guide (7 Days)</v>
-      </c>
-      <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>150</v>
+        <v>☐</v>
+      </c>
+      <c r="D2" t="str">
+        <v>☐</v>
+      </c>
+      <c r="E2" t="str">
+        <v>☑</v>
       </c>
       <c r="F2">
-        <v>1050</v>
+        <v>250</v>
+      </c>
+      <c r="G2">
+        <v>27</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>7000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BVP05072026</v>
+        <v>CityTax</v>
       </c>
       <c r="B3" t="str">
-        <v>Transport</v>
+        <v>☐</v>
       </c>
       <c r="C3" t="str">
-        <v>Luxury Bus Budapest-Vienna-Prague</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>3200</v>
+        <v>☑</v>
+      </c>
+      <c r="D3" t="str">
+        <v>☐</v>
+      </c>
+      <c r="E3" t="str">
+        <v>☑</v>
       </c>
       <c r="F3">
-        <v>3200</v>
+        <v>2.5</v>
+      </c>
+      <c r="G3">
+        <v>27</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>435</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>